<commit_message>
atualização mensal da planilha
</commit_message>
<xml_diff>
--- a/Valor mensal Tibia - 2026.xlsx
+++ b/Valor mensal Tibia - 2026.xlsx
@@ -19,7 +19,7 @@
     <sheet state="visible" name="Dezembro" sheetId="14" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Extrato R$'!$B$3:$G$48</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Extrato R$'!$B$3:$G$71</definedName>
     <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">Janeiro!$B$6:$J$37</definedName>
     <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">Fevereiro!$B$6:$J$34</definedName>
     <definedName hidden="1" localSheetId="4" name="_xlnm._FilterDatabase">'Março'!$B$6:$J$37</definedName>
@@ -40,11 +40,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={6ee2dd78-5128-4080-99be-0b5c9cd41edf}</author>
-    <author>tc={cf4f9192-cea5-44d8-8dfe-e102742654bf}</author>
+    <author>tc={b18cd86b-d04d-4fb4-ba21-954fcff7aaf4}</author>
+    <author>tc={c802b1f9-854c-4952-be8a-4359bb30a356}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{6ee2dd78-5128-4080-99be-0b5c9cd41edf}" ref="A1">
+    <comment authorId="0" xr:uid="{b18cd86b-d04d-4fb4-ba21-954fcff7aaf4}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -53,7 +53,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{cf4f9192-cea5-44d8-8dfe-e102742654bf}" ref="A1">
+    <comment authorId="1" xr:uid="{c802b1f9-854c-4952-be8a-4359bb30a356}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -69,15 +69,33 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={44853ffe-1b41-4859-859b-bf1f6d24b685}</author>
-    <author>tc={456b592e-293b-4dcc-9d2c-599f75e4e8e0}</author>
-    <author>tc={697e73a9-281b-4164-8e96-8c3c24f374c4}</author>
-    <author>tc={8cb99176-8156-4650-86cd-4475a19089c4}</author>
-    <author>tc={b2b1c725-a1e3-491f-8e2e-89ddb63bb0f3}</author>
-    <author>tc={fc8b6505-28d6-4f42-b2ae-cf52f839157d}</author>
+    <author>tc={80eed69c-a5a6-453f-bcdb-a18e29b87e77}</author>
+    <author>tc={80faf8d3-5585-4da4-9870-a9bdb265a67c}</author>
+    <author>tc={8ac2462c-b473-4989-9293-19b3a327d37d}</author>
+    <author>tc={aaa872a2-c68e-42ab-83ba-831d082cf545}</author>
+    <author>tc={b765600f-e2ca-4201-ab27-07b7c46b2e18}</author>
+    <author>tc={ecfa7a82-7797-40a8-8989-65d79fbe1671}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{44853ffe-1b41-4859-859b-bf1f6d24b685}" ref="D5">
+    <comment authorId="0" xr:uid="{80eed69c-a5a6-453f-bcdb-a18e29b87e77}" ref="L8">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Uso média apenas onde analiso volume, e mediana onde preciso decidir.
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{80faf8d3-5585-4da4-9870-a9bdb265a67c}" ref="U7">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Mediana utilizada na fórmula de formatação condicional para evitar valores exagerados devido a drops raros, mantendo assim valores reais
+</t>
+      </text>
+    </comment>
+    <comment authorId="2" xr:uid="{8ac2462c-b473-4989-9293-19b3a327d37d}" ref="D5">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -86,7 +104,25 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{456b592e-293b-4dcc-9d2c-599f75e4e8e0}" ref="C6">
+    <comment authorId="3" xr:uid="{aaa872a2-c68e-42ab-83ba-831d082cf545}" ref="L9">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Mediana utilizada para evitar valores exagerados devido a drops raros, mantendo assim valores reais
+</t>
+      </text>
+    </comment>
+    <comment authorId="4" xr:uid="{b765600f-e2ca-4201-ab27-07b7c46b2e18}" ref="H6">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	TC teórico, sem o uso de múltiplo de 25 para evitar arrendondamentos e consequentemente perda de dados
+</t>
+      </text>
+    </comment>
+    <comment authorId="5" xr:uid="{ecfa7a82-7797-40a8-8989-65d79fbe1671}" ref="C6">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,48 +131,12 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{697e73a9-281b-4164-8e96-8c3c24f374c4}" ref="L8">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Uso média apenas onde analiso volume, e mediana onde preciso decidir.
-</t>
-      </text>
-    </comment>
-    <comment authorId="3" xr:uid="{8cb99176-8156-4650-86cd-4475a19089c4}" ref="U7">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Mediana utilizada na fórmula de formatação condicional para evitar valores exagerados devido a drops raros, mantendo assim valores reais
-</t>
-      </text>
-    </comment>
-    <comment authorId="4" xr:uid="{b2b1c725-a1e3-491f-8e2e-89ddb63bb0f3}" ref="H6">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	TC teórico, sem o uso de múltiplo de 25 para evitar arrendondamentos e consequentemente perda de dados
-</t>
-      </text>
-    </comment>
-    <comment authorId="5" xr:uid="{fc8b6505-28d6-4f42-b2ae-cf52f839157d}" ref="L9">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Mediana utilizada para evitar valores exagerados devido a drops raros, mantendo assim valores reais
-</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="65">
   <si>
     <t>Coin Mediana</t>
   </si>
@@ -939,7 +939,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Joao Vitor (Clovis)" id="{c1782948-1944-4d9b-8cb5-900612da6168}" providerId="google-sheets"/>
+  <x18tc:person displayName="Joao Vitor (Clovis)" id="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1139,10 +1139,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A1" dT="2026-01-04T19:55:45.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{6ee2dd78-5128-4080-99be-0b5c9cd41edf}" done="1">
+  <x18tc:threadedComment ref="A1" dT="2026-01-04T19:55:45.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{b18cd86b-d04d-4fb4-ba21-954fcff7aaf4}" done="1">
     <x18tc:text xml:space="preserve">Arcans Sunrise</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-01-04T19:55:13.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{cf4f9192-cea5-44d8-8dfe-e102742654bf}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-01-04T19:55:13.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{c802b1f9-854c-4952-be8a-4359bb30a356}" done="0">
     <x18tc:text xml:space="preserve">Itz Megan</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1150,22 +1150,22 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="L9" dT="2026-01-04T19:54:20.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{fc8b6505-28d6-4f42-b2ae-cf52f839157d}" done="1">
+  <x18tc:threadedComment ref="L9" dT="2026-01-04T19:54:20.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{aaa872a2-c68e-42ab-83ba-831d082cf545}" done="1">
     <x18tc:text xml:space="preserve">Mediana utilizada para evitar valores exagerados devido a drops raros, mantendo assim valores reais</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="C6" dT="2026-01-05T19:28:58.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{456b592e-293b-4dcc-9d2c-599f75e4e8e0}" done="1">
+  <x18tc:threadedComment ref="C6" dT="2026-01-05T19:28:58.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{ecfa7a82-7797-40a8-8989-65d79fbe1671}" done="1">
     <x18tc:text xml:space="preserve">O valor do Tibia Coin utilizado é o menor preço entre as ofertas com maior volume disponível, priorizando liquidez e evitando ruídos ou valores não representativos do mercado.</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="H6" dT="2026-01-04T19:52:38.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{b2b1c725-a1e3-491f-8e2e-89ddb63bb0f3}" done="1">
+  <x18tc:threadedComment ref="H6" dT="2026-01-04T19:52:38.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{b765600f-e2ca-4201-ab27-07b7c46b2e18}" done="1">
     <x18tc:text xml:space="preserve">TC teórico, sem o uso de múltiplo de 25 para evitar arrendondamentos e consequentemente perda de dados</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="D5" dT="2026-01-04T19:55:30.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{44853ffe-1b41-4859-859b-bf1f6d24b685}" done="1">
+  <x18tc:threadedComment ref="D5" dT="2026-01-04T19:55:30.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{8ac2462c-b473-4989-9293-19b3a327d37d}" done="1">
     <x18tc:text xml:space="preserve">Itz Megan</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L8" dT="2026-01-06T02:05:26.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{697e73a9-281b-4164-8e96-8c3c24f374c4}" done="1">
+  <x18tc:threadedComment ref="L8" dT="2026-01-06T02:05:26.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{80eed69c-a5a6-453f-bcdb-a18e29b87e77}" done="1">
     <x18tc:text xml:space="preserve">Uso média apenas onde analiso volume, e mediana onde preciso decidir.</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="U7" dT="2026-01-04T20:05:30.00" personId="{c1782948-1944-4d9b-8cb5-900612da6168}" id="{8cb99176-8156-4650-86cd-4475a19089c4}" done="1">
+  <x18tc:threadedComment ref="U7" dT="2026-01-04T20:05:30.00" personId="{d5d2cef1-df46-4ee6-804f-ee2bfa2e6b1b}" id="{80faf8d3-5585-4da4-9870-a9bdb265a67c}" done="1">
     <x18tc:text xml:space="preserve">Mediana utilizada na fórmula de formatação condicional para evitar valores exagerados devido a drops raros, mantendo assim valores reais</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1347,47 +1347,47 @@
       </c>
       <c r="C5" s="13">
         <f>'Março'!$M$8</f>
-        <v>38949</v>
+        <v>38498</v>
       </c>
       <c r="D5" s="14">
         <f>'Março'!$M$10</f>
-        <v>23546568</v>
+        <v>208999761</v>
       </c>
       <c r="E5" s="14">
         <f>'Março'!$M$9</f>
-        <v>8861162</v>
+        <v>7255621</v>
       </c>
       <c r="F5" s="14">
         <f t="shared" si="1"/>
-        <v>7848856</v>
+        <v>6741927.774</v>
       </c>
       <c r="G5" s="14">
         <f>IFERROR(AVERAGE('Março'!$D$7:$D$37), 0)</f>
-        <v>3422978</v>
+        <v>3988847.032</v>
       </c>
       <c r="H5" s="14">
         <f>IFERROR(AVERAGE('Março'!$E$7:$E$37), 0)</f>
-        <v>2138652.25</v>
+        <v>2675594.871</v>
       </c>
       <c r="I5" s="14">
         <f>IFERROR(AVERAGE('Março'!$F$7:$F$37), 0)</f>
-        <v>325011.75</v>
+        <v>77485.87097</v>
       </c>
       <c r="J5" s="15" t="str">
         <f>if('Março'!$R$13 = "🔵 Concluído","Ok", "No")</f>
-        <v>No</v>
+        <v>Ok</v>
       </c>
       <c r="K5" s="16">
         <f>IFERROR(D5/'Março'!$M$11, 0)</f>
-        <v>0.1209097435</v>
+        <v>1.085769448</v>
       </c>
       <c r="L5" s="15">
         <f>'Março'!$R$9</f>
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="M5" s="17">
         <f>'Março'!$R$11</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1395,9 +1395,9 @@
       <c r="B6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="13" t="str">
+      <c r="C6" s="13">
         <f>Abril!$M$8</f>
-        <v/>
+        <v>38396</v>
       </c>
       <c r="D6" s="14">
         <f>Abril!$M$10</f>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="J6" s="15" t="str">
         <f>if(Abril!$R$13 = "🔵 Concluído","Ok", "No")</f>
-        <v>Ok</v>
+        <v>No</v>
       </c>
       <c r="K6" s="16">
         <f>IFERROR(D6/Abril!$M$11, 0)</f>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="M6" s="17">
         <f>Abril!$R$11</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -31893,7 +31893,7 @@
         <v>46024.0</v>
       </c>
       <c r="C4" s="40" t="str">
-        <f t="shared" ref="C4:C48" si="1">(TEXT(B4,"mm/yyyy"))</f>
+        <f t="shared" ref="C4:C71" si="1">(TEXT(B4,"mm/yyyy"))</f>
         <v>01/2026</v>
       </c>
       <c r="D4" s="41" t="s">
@@ -31906,7 +31906,7 @@
         <v>53.5</v>
       </c>
       <c r="G4" s="43">
-        <f t="shared" ref="G4:G48" si="2"> E4/250 * F4</f>
+        <f t="shared" ref="G4:G71" si="2"> E4/250 * F4</f>
         <v>21.4</v>
       </c>
       <c r="I4" s="44" t="s">
@@ -32024,30 +32024,30 @@
       <c r="J6" s="50">
         <f>SUMIFS($E$4:$E1003,$C$4:$C1003,"2026-03",$D$4:$D1003,"Compra")
 </f>
-        <v>375</v>
+        <v>4850</v>
       </c>
       <c r="K6" s="51">
         <f>SUMIFS($E$4:$E1003,$C$4:$C1003,"2026-03",$D$4:$D1003,"Uso")
 </f>
-        <v>0</v>
+        <v>2725</v>
       </c>
       <c r="L6" s="51">
         <f>SUMIFS($E$4:$E1003,$C$4:$C1003,"2026-03",$D$4:$D1003,"Venda")
 </f>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="M6" s="51">
         <f t="shared" si="4"/>
-        <v>1750</v>
+        <v>500</v>
       </c>
       <c r="N6" s="52">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(MEDIAN(FILTER($F$4:$F1003,$C$4:$C1003=""03/2026"",$D$4:$D1003=""Compra""), ), 0
-)"),52.0)</f>
-        <v>52</v>
+)"),51.0)</f>
+        <v>51</v>
       </c>
       <c r="O6" s="53">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>612</v>
       </c>
     </row>
     <row r="7">
@@ -33349,210 +33349,532 @@
     </row>
     <row r="49">
       <c r="A49" s="64"/>
-      <c r="B49" s="64"/>
-      <c r="C49" s="67"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="52"/>
-      <c r="G49" s="55"/>
+      <c r="B49" s="39">
+        <v>46085.0</v>
+      </c>
+      <c r="C49" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D49" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E49" s="42">
+        <v>375.0</v>
+      </c>
+      <c r="F49" s="41">
+        <v>52.0</v>
+      </c>
+      <c r="G49" s="43">
+        <f t="shared" si="2"/>
+        <v>78</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="64"/>
-      <c r="B50" s="64"/>
-      <c r="C50" s="67"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="56"/>
-      <c r="F50" s="52"/>
-      <c r="G50" s="55"/>
+      <c r="B50" s="39">
+        <v>46086.0</v>
+      </c>
+      <c r="C50" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D50" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E50" s="42">
+        <v>125.0</v>
+      </c>
+      <c r="F50" s="41">
+        <v>52.0</v>
+      </c>
+      <c r="G50" s="43">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="64"/>
-      <c r="B51" s="64"/>
-      <c r="C51" s="67"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="52"/>
-      <c r="G51" s="55"/>
+      <c r="B51" s="39">
+        <v>46087.0</v>
+      </c>
+      <c r="C51" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D51" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E51" s="42">
+        <v>125.0</v>
+      </c>
+      <c r="F51" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G51" s="43">
+        <f t="shared" si="2"/>
+        <v>25.5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="64"/>
-      <c r="B52" s="64"/>
-      <c r="C52" s="67"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="56"/>
-      <c r="F52" s="52"/>
-      <c r="G52" s="55"/>
+      <c r="B52" s="39">
+        <v>46088.0</v>
+      </c>
+      <c r="C52" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D52" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E52" s="42">
+        <v>125.0</v>
+      </c>
+      <c r="F52" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G52" s="43">
+        <f t="shared" si="2"/>
+        <v>25.5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="64"/>
-      <c r="B53" s="64"/>
-      <c r="C53" s="67"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="56"/>
-      <c r="F53" s="52"/>
-      <c r="G53" s="55"/>
+      <c r="B53" s="39">
+        <v>46088.0</v>
+      </c>
+      <c r="C53" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D53" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E53" s="42">
+        <v>400.0</v>
+      </c>
+      <c r="F53" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G53" s="43">
+        <f t="shared" si="2"/>
+        <v>81.6</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="64"/>
-      <c r="B54" s="64"/>
-      <c r="C54" s="67"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="56"/>
-      <c r="F54" s="52"/>
-      <c r="G54" s="55"/>
+      <c r="B54" s="39">
+        <v>46090.0</v>
+      </c>
+      <c r="C54" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D54" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E54" s="42">
+        <v>150.0</v>
+      </c>
+      <c r="F54" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G54" s="43">
+        <f t="shared" si="2"/>
+        <v>30.6</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="64"/>
-      <c r="B55" s="64"/>
-      <c r="C55" s="67"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="55"/>
+      <c r="B55" s="39">
+        <v>46091.0</v>
+      </c>
+      <c r="C55" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D55" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E55" s="42">
+        <v>250.0</v>
+      </c>
+      <c r="F55" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G55" s="43">
+        <f t="shared" si="2"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="64"/>
-      <c r="B56" s="64"/>
-      <c r="C56" s="67"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="56"/>
-      <c r="F56" s="52"/>
-      <c r="G56" s="55"/>
+      <c r="B56" s="39">
+        <v>46092.0</v>
+      </c>
+      <c r="C56" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D56" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E56" s="42">
+        <v>250.0</v>
+      </c>
+      <c r="F56" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G56" s="43">
+        <f t="shared" si="2"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="64"/>
-      <c r="B57" s="64"/>
-      <c r="C57" s="67"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="56"/>
-      <c r="F57" s="52"/>
-      <c r="G57" s="55"/>
+      <c r="B57" s="66">
+        <v>46093.0</v>
+      </c>
+      <c r="C57" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D57" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E57" s="42">
+        <v>100.0</v>
+      </c>
+      <c r="F57" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G57" s="43">
+        <f t="shared" si="2"/>
+        <v>20.4</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="64"/>
-      <c r="B58" s="64"/>
-      <c r="C58" s="67"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="55"/>
+      <c r="B58" s="39">
+        <v>46093.0</v>
+      </c>
+      <c r="C58" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D58" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E58" s="42">
+        <v>1025.0</v>
+      </c>
+      <c r="F58" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G58" s="43">
+        <f t="shared" si="2"/>
+        <v>209.1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="64"/>
-      <c r="B59" s="64"/>
-      <c r="C59" s="67"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="56"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="55"/>
+      <c r="B59" s="39">
+        <v>46094.0</v>
+      </c>
+      <c r="C59" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D59" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E59" s="42">
+        <v>200.0</v>
+      </c>
+      <c r="F59" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G59" s="43">
+        <f t="shared" si="2"/>
+        <v>40.8</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="64"/>
-      <c r="B60" s="64"/>
-      <c r="C60" s="67"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="56"/>
-      <c r="F60" s="52"/>
-      <c r="G60" s="55"/>
+      <c r="B60" s="39">
+        <v>46096.0</v>
+      </c>
+      <c r="C60" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D60" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E60" s="42">
+        <v>250.0</v>
+      </c>
+      <c r="F60" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G60" s="43">
+        <f t="shared" si="2"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="64"/>
-      <c r="B61" s="64"/>
-      <c r="C61" s="67"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="56"/>
-      <c r="F61" s="52"/>
-      <c r="G61" s="55"/>
+      <c r="B61" s="39">
+        <v>46098.0</v>
+      </c>
+      <c r="C61" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D61" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E61" s="42">
+        <v>125.0</v>
+      </c>
+      <c r="F61" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G61" s="43">
+        <f t="shared" si="2"/>
+        <v>25.5</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="64"/>
-      <c r="B62" s="64"/>
-      <c r="C62" s="67"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="56"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="55"/>
+      <c r="B62" s="39">
+        <v>46099.0</v>
+      </c>
+      <c r="C62" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D62" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E62" s="42">
+        <v>500.0</v>
+      </c>
+      <c r="F62" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G62" s="43">
+        <f t="shared" si="2"/>
+        <v>102</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="64"/>
-      <c r="B63" s="64"/>
-      <c r="C63" s="67"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="56"/>
-      <c r="F63" s="52"/>
-      <c r="G63" s="55"/>
+      <c r="B63" s="39">
+        <v>46102.0</v>
+      </c>
+      <c r="C63" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D63" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E63" s="42">
+        <v>1100.0</v>
+      </c>
+      <c r="F63" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G63" s="43">
+        <f t="shared" si="2"/>
+        <v>224.4</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="64"/>
-      <c r="B64" s="64"/>
-      <c r="C64" s="67"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="56"/>
-      <c r="F64" s="52"/>
-      <c r="G64" s="55"/>
+      <c r="B64" s="39">
+        <v>46102.0</v>
+      </c>
+      <c r="C64" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D64" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E64" s="42">
+        <v>100.0</v>
+      </c>
+      <c r="F64" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G64" s="43">
+        <f t="shared" si="2"/>
+        <v>20.4</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="64"/>
-      <c r="B65" s="64"/>
-      <c r="C65" s="67"/>
-      <c r="D65" s="14"/>
-      <c r="E65" s="56"/>
-      <c r="F65" s="52"/>
-      <c r="G65" s="55"/>
+      <c r="B65" s="39">
+        <v>46102.0</v>
+      </c>
+      <c r="C65" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D65" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E65" s="42">
+        <v>250.0</v>
+      </c>
+      <c r="F65" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G65" s="43">
+        <f t="shared" si="2"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="64"/>
-      <c r="B66" s="64"/>
-      <c r="C66" s="67"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="56"/>
-      <c r="F66" s="52"/>
-      <c r="G66" s="55"/>
+      <c r="B66" s="39">
+        <v>46102.0</v>
+      </c>
+      <c r="C66" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D66" s="41" t="s">
+        <v>39</v>
+      </c>
+      <c r="E66" s="42">
+        <v>1500.0</v>
+      </c>
+      <c r="F66" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G66" s="43">
+        <f t="shared" si="2"/>
+        <v>306</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="64"/>
-      <c r="B67" s="64"/>
-      <c r="C67" s="67"/>
-      <c r="D67" s="14"/>
-      <c r="E67" s="56"/>
-      <c r="F67" s="52"/>
-      <c r="G67" s="55"/>
+      <c r="B67" s="39">
+        <v>46105.0</v>
+      </c>
+      <c r="C67" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D67" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E67" s="42">
+        <v>500.0</v>
+      </c>
+      <c r="F67" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G67" s="43">
+        <f t="shared" si="2"/>
+        <v>102</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="64"/>
-      <c r="B68" s="64"/>
-      <c r="C68" s="67"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="56"/>
-      <c r="F68" s="52"/>
-      <c r="G68" s="55"/>
+      <c r="B68" s="39">
+        <v>46106.0</v>
+      </c>
+      <c r="C68" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D68" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E68" s="42">
+        <v>250.0</v>
+      </c>
+      <c r="F68" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G68" s="43">
+        <f t="shared" si="2"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="64"/>
-      <c r="B69" s="64"/>
-      <c r="C69" s="67"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="56"/>
-      <c r="F69" s="52"/>
-      <c r="G69" s="55"/>
+      <c r="B69" s="39">
+        <v>46109.0</v>
+      </c>
+      <c r="C69" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D69" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E69" s="42">
+        <v>500.0</v>
+      </c>
+      <c r="F69" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G69" s="43">
+        <f t="shared" si="2"/>
+        <v>102</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="64"/>
-      <c r="B70" s="64"/>
-      <c r="C70" s="67"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="56"/>
-      <c r="F70" s="52"/>
-      <c r="G70" s="55"/>
+      <c r="B70" s="39">
+        <v>46109.0</v>
+      </c>
+      <c r="C70" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D70" s="41" t="s">
+        <v>39</v>
+      </c>
+      <c r="E70" s="42">
+        <v>1500.0</v>
+      </c>
+      <c r="F70" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G70" s="43">
+        <f t="shared" si="2"/>
+        <v>306</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="64"/>
-      <c r="B71" s="64"/>
-      <c r="C71" s="67"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="56"/>
-      <c r="F71" s="52"/>
-      <c r="G71" s="55"/>
+      <c r="B71" s="39">
+        <v>46112.0</v>
+      </c>
+      <c r="C71" s="40" t="str">
+        <f t="shared" si="1"/>
+        <v>03/2026</v>
+      </c>
+      <c r="D71" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E71" s="42">
+        <v>500.0</v>
+      </c>
+      <c r="F71" s="41">
+        <v>51.0</v>
+      </c>
+      <c r="G71" s="43">
+        <f t="shared" si="2"/>
+        <v>102</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="64"/>
@@ -41943,13 +42265,13 @@
       <c r="G1003" s="55"/>
     </row>
   </sheetData>
-  <autoFilter ref="$B$3:$G$48"/>
+  <autoFilter ref="$B$3:$G$71"/>
   <mergeCells count="2">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="J2:O2"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4:D48">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D4:D71">
       <formula1>"Venda,Compra,Uso"</formula1>
     </dataValidation>
   </dataValidations>
@@ -54536,7 +54858,7 @@
         <v>41</v>
       </c>
       <c r="C3" s="70">
-        <v>52.0</v>
+        <v>51.0</v>
       </c>
       <c r="J3" s="15"/>
       <c r="V3" s="15"/>
@@ -54625,12 +54947,12 @@
         <v>5726484</v>
       </c>
       <c r="H7" s="76">
-        <f t="shared" ref="H7:H34" si="2">IFERROR(G7/C7, )</f>
+        <f t="shared" ref="H7:H37" si="2">IFERROR(G7/C7, )</f>
         <v>148.3545078</v>
       </c>
       <c r="I7" s="77">
         <f t="shared" ref="I7:I37" si="3">IFERROR(H7/25 * ($C$3/10), )</f>
-        <v>30.85773762</v>
+        <v>30.26431959</v>
       </c>
       <c r="J7" s="41" t="str">
         <f t="shared" ref="J7:J37" si="4">IF(B7 &gt; TODAY(), "", IF(G7 = "", "Não", "Sim"))
@@ -54687,7 +55009,7 @@
       </c>
       <c r="I8" s="77">
         <f t="shared" si="3"/>
-        <v>46.90115772</v>
+        <v>45.99921238</v>
       </c>
       <c r="J8" s="41" t="str">
         <f t="shared" si="4"/>
@@ -54698,7 +55020,7 @@
       </c>
       <c r="M8" s="85">
         <f> IFERROR(MEDIAN(C7:C999), )</f>
-        <v>38949</v>
+        <v>38498</v>
       </c>
       <c r="N8" s="86"/>
       <c r="O8" s="87"/>
@@ -54746,7 +55068,7 @@
       </c>
       <c r="I9" s="77">
         <f t="shared" si="3"/>
-        <v>46.71720257</v>
+        <v>45.81879483</v>
       </c>
       <c r="J9" s="41" t="str">
         <f t="shared" si="4"/>
@@ -54757,15 +55079,15 @@
       </c>
       <c r="M9" s="56">
         <f t="shared" ref="M9:N9" si="5"> IFERROR(MEDIAN(G7:G999), )</f>
-        <v>8861162</v>
+        <v>7255621</v>
       </c>
       <c r="N9" s="56">
         <f t="shared" si="5"/>
-        <v>186.4782216</v>
+        <v>190.6980158</v>
       </c>
       <c r="O9" s="93">
         <f> IFERROR($N$9 * ($C$3/10)  / 25, )</f>
-        <v>38.78747009</v>
+        <v>38.90239521</v>
       </c>
       <c r="P9" s="88"/>
       <c r="Q9" s="89" t="s">
@@ -54773,7 +55095,7 @@
       </c>
       <c r="R9" s="17">
         <f>COUNTIF(J:J, "=Sim")</f>
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="T9" s="90"/>
       <c r="U9" s="91"/>
@@ -54788,47 +55110,49 @@
         <v>46085.0</v>
       </c>
       <c r="C10" s="75">
-        <v>38488.0</v>
+        <v>37949.0</v>
       </c>
       <c r="D10" s="75">
-        <v>0.0</v>
+        <f> 2889635 + 1585814</f>
+        <v>4475449</v>
       </c>
       <c r="E10" s="75">
-        <v>0.0</v>
+        <f> 1684132 + 1077218</f>
+        <v>2761350</v>
       </c>
       <c r="F10" s="75">
         <v>0.0</v>
       </c>
-      <c r="G10" s="56" t="str">
+      <c r="G10" s="56">
         <f t="shared" si="1"/>
-        <v/>
+        <v>7236799</v>
       </c>
       <c r="H10" s="76">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>190.6980158</v>
       </c>
       <c r="I10" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>38.90239521</v>
       </c>
       <c r="J10" s="41" t="str">
         <f t="shared" si="4"/>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="L10" s="89" t="s">
         <v>59</v>
       </c>
       <c r="M10" s="94">
         <f>IFERROR(SUM(G7:G999), )</f>
-        <v>23546568</v>
+        <v>208999761</v>
       </c>
       <c r="N10" s="95">
         <f> IFERROR($M$10 / $M$8, )</f>
-        <v>604.5487176</v>
+        <v>5428.847239</v>
       </c>
       <c r="O10" s="93">
         <f> IFERROR($N$10 * ($C$3/10)  / 25, )</f>
-        <v>125.7461333</v>
+        <v>1107.484837</v>
       </c>
       <c r="P10" s="88"/>
       <c r="Q10" s="89" t="s">
@@ -54836,7 +55160,7 @@
       </c>
       <c r="R10" s="96">
         <f>IFERROR(M12/M9, )</f>
-        <v>19.32008827</v>
+        <v>-2.275444238</v>
       </c>
       <c r="T10" s="90"/>
       <c r="U10" s="91"/>
@@ -54850,32 +55174,42 @@
       <c r="B11" s="39">
         <v>46086.0</v>
       </c>
-      <c r="C11" s="75"/>
-      <c r="D11" s="75"/>
-      <c r="E11" s="75"/>
-      <c r="F11" s="75"/>
-      <c r="G11" s="56" t="str">
+      <c r="C11" s="75">
+        <v>37900.0</v>
+      </c>
+      <c r="D11" s="75">
+        <f> 1370867 + 1359419 + 1500000</f>
+        <v>4230286</v>
+      </c>
+      <c r="E11" s="75">
+        <f> 1870522 + 1180452</f>
+        <v>3050974</v>
+      </c>
+      <c r="F11" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H11" s="76" t="str">
+        <v>7281260</v>
+      </c>
+      <c r="H11" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>192.1176781</v>
       </c>
       <c r="I11" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>39.19200633</v>
       </c>
       <c r="J11" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="L11" s="89" t="s">
         <v>61</v>
       </c>
       <c r="M11" s="75">
         <f> IFERROR($N$11 * $M$8, )</f>
-        <v>194745000</v>
+        <v>192490000</v>
       </c>
       <c r="N11" s="98">
         <f> IFERROR($C$4, )</f>
@@ -54883,14 +55217,14 @@
       </c>
       <c r="O11" s="93">
         <f> IFERROR($N$11 * ($C$3/10)  / 25,"")</f>
-        <v>1040</v>
+        <v>1020</v>
       </c>
       <c r="Q11" s="89" t="s">
         <v>62</v>
       </c>
       <c r="R11" s="17">
         <f>COUNTIF($J:$J, "=Não")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T11" s="90"/>
       <c r="U11" s="91"/>
@@ -54901,50 +55235,59 @@
     </row>
     <row r="12">
       <c r="A12" s="39"/>
-      <c r="B12" s="39">
+      <c r="B12" s="103">
         <v>46087.0</v>
       </c>
-      <c r="C12" s="75"/>
-      <c r="D12" s="75"/>
-      <c r="E12" s="56"/>
-      <c r="F12" s="75"/>
-      <c r="G12" s="56" t="str">
+      <c r="C12" s="75">
+        <v>38993.0</v>
+      </c>
+      <c r="D12" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="E12" s="75">
+        <f> 944578 + 1211390 + 858872</f>
+        <v>3014840</v>
+      </c>
+      <c r="F12" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G12" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H12" s="76" t="str">
+        <v>3014840</v>
+      </c>
+      <c r="H12" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>77.31746724</v>
       </c>
       <c r="I12" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>15.77276332</v>
       </c>
       <c r="J12" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="L12" s="89" t="s">
         <v>63</v>
       </c>
       <c r="M12" s="56">
         <f> IFERROR($M$11 - $M$10, )</f>
-        <v>171198432</v>
+        <v>-16509761</v>
       </c>
       <c r="N12" s="56">
         <f>N11 - N10</f>
-        <v>4395.451282</v>
+        <v>-428.8472388</v>
       </c>
       <c r="O12" s="93">
         <f> IFERROR($N$12 * ($C$3/10)  / 25, )</f>
-        <v>914.2538667</v>
+        <v>-87.48483672</v>
       </c>
       <c r="Q12" s="89" t="s">
         <v>64</v>
       </c>
       <c r="R12" s="96">
         <f>R8 - R9 - R10</f>
-        <v>8.679911732</v>
+        <v>2.275444238</v>
       </c>
       <c r="T12" s="90"/>
       <c r="U12" s="91"/>
@@ -54955,28 +55298,38 @@
     </row>
     <row r="13">
       <c r="A13" s="39"/>
-      <c r="B13" s="39">
+      <c r="B13" s="103">
         <v>46088.0</v>
       </c>
-      <c r="C13" s="75"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
-      <c r="F13" s="75"/>
-      <c r="G13" s="56" t="str">
+      <c r="C13" s="75">
+        <v>38099.0</v>
+      </c>
+      <c r="D13" s="75">
+        <f> 296185 + 86358 + 408589</f>
+        <v>791132</v>
+      </c>
+      <c r="E13" s="75">
+        <f> 1263502 + 509101 + 1230129</f>
+        <v>3002732</v>
+      </c>
+      <c r="F13" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G13" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H13" s="76" t="str">
+        <v>3793864</v>
+      </c>
+      <c r="H13" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>99.57909656</v>
       </c>
       <c r="I13" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>20.3141357</v>
       </c>
       <c r="J13" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="L13" s="99"/>
       <c r="M13" s="100"/>
@@ -54987,7 +55340,7 @@
       </c>
       <c r="R13" s="23" t="str">
         <f>IF(M10 &gt;= M11, "🔵 Concluído", IF((R8-R9)-R10-R11&gt;=2, "🟢 Seguro", IF((R8-R9)-R10-R11&gt;=0, "🟡 Atenção", "🔴 Risco")))</f>
-        <v>🟢 Seguro</v>
+        <v>🔵 Concluído</v>
       </c>
       <c r="T13" s="90"/>
       <c r="U13" s="91"/>
@@ -54998,28 +55351,38 @@
     </row>
     <row r="14">
       <c r="A14" s="39"/>
-      <c r="B14" s="39">
+      <c r="B14" s="103">
         <v>46089.0</v>
       </c>
-      <c r="C14" s="75"/>
-      <c r="D14" s="75"/>
-      <c r="E14" s="75"/>
-      <c r="F14" s="75"/>
-      <c r="G14" s="56" t="str">
+      <c r="C14" s="75">
+        <v>38095.0</v>
+      </c>
+      <c r="D14" s="75">
+        <f> 1287862 + 1627561</f>
+        <v>2915423</v>
+      </c>
+      <c r="E14" s="75">
+        <f> 1959894 + 952496 + 92467</f>
+        <v>3004857</v>
+      </c>
+      <c r="F14" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G14" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H14" s="76" t="str">
+        <v>5920280</v>
+      </c>
+      <c r="H14" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>155.4083213</v>
       </c>
       <c r="I14" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>31.70329755</v>
       </c>
       <c r="J14" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -55036,25 +55399,35 @@
       <c r="B15" s="39">
         <v>46090.0</v>
       </c>
-      <c r="C15" s="75"/>
-      <c r="D15" s="75"/>
-      <c r="E15" s="75"/>
-      <c r="F15" s="75"/>
-      <c r="G15" s="56" t="str">
+      <c r="C15" s="75">
+        <v>38498.0</v>
+      </c>
+      <c r="D15" s="75">
+        <f> 2611132 + 1217971 + 1744899 + 247550 + 704766</f>
+        <v>6526318</v>
+      </c>
+      <c r="E15" s="75">
+        <f> 1826907 + 1209214</f>
+        <v>3036121</v>
+      </c>
+      <c r="F15" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G15" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H15" s="76" t="str">
+        <v>9562439</v>
+      </c>
+      <c r="H15" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>248.3879422</v>
       </c>
       <c r="I15" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>50.67114022</v>
       </c>
       <c r="J15" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="L15" s="1"/>
       <c r="V15" s="15"/>
@@ -55065,25 +55438,35 @@
       <c r="B16" s="39">
         <v>46091.0</v>
       </c>
-      <c r="C16" s="75"/>
-      <c r="D16" s="75"/>
-      <c r="E16" s="75"/>
-      <c r="F16" s="75"/>
-      <c r="G16" s="56" t="str">
+      <c r="C16" s="75">
+        <v>38198.0</v>
+      </c>
+      <c r="D16" s="75">
+        <f> 2126989</f>
+        <v>2126989</v>
+      </c>
+      <c r="E16" s="75">
+        <f> 1795121 + 945185</f>
+        <v>2740306</v>
+      </c>
+      <c r="F16" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G16" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H16" s="76" t="str">
+        <v>4867295</v>
+      </c>
+      <c r="H16" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>127.4227708</v>
       </c>
       <c r="I16" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>25.99424525</v>
       </c>
       <c r="J16" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="N16" s="102"/>
       <c r="V16" s="15"/>
@@ -55094,25 +55477,35 @@
       <c r="B17" s="39">
         <v>46092.0</v>
       </c>
-      <c r="C17" s="75"/>
-      <c r="D17" s="75"/>
-      <c r="E17" s="75"/>
-      <c r="F17" s="75"/>
-      <c r="G17" s="56" t="str">
+      <c r="C17" s="75">
+        <v>38196.0</v>
+      </c>
+      <c r="D17" s="75">
+        <f> 1821921 - 130627 + 2605544 + 1388582</f>
+        <v>5685420</v>
+      </c>
+      <c r="E17" s="75">
+        <f> 1586198 + 546884</f>
+        <v>2133082</v>
+      </c>
+      <c r="F17" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G17" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H17" s="76" t="str">
+        <v>7818502</v>
+      </c>
+      <c r="H17" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>204.6942612</v>
       </c>
       <c r="I17" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>41.75762928</v>
       </c>
       <c r="J17" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V17" s="15"/>
       <c r="W17" s="15"/>
@@ -55122,25 +55515,35 @@
       <c r="B18" s="39">
         <v>46093.0</v>
       </c>
-      <c r="C18" s="56"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56" t="str">
+      <c r="C18" s="75">
+        <v>38193.0</v>
+      </c>
+      <c r="D18" s="75">
+        <f> 1910486 + 913030 + 1527523 + 536720 + 720150 + 426128</f>
+        <v>6034037</v>
+      </c>
+      <c r="E18" s="75">
+        <f> 2026332 + 1024892</f>
+        <v>3051224</v>
+      </c>
+      <c r="F18" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G18" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H18" s="76" t="str">
+        <v>9085261</v>
+      </c>
+      <c r="H18" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>237.8776477</v>
       </c>
       <c r="I18" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>48.52704014</v>
       </c>
       <c r="J18" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V18" s="15"/>
       <c r="W18" s="15"/>
@@ -55150,25 +55553,35 @@
       <c r="B19" s="39">
         <v>46094.0</v>
       </c>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56" t="str">
+      <c r="C19" s="75">
+        <v>38099.0</v>
+      </c>
+      <c r="D19" s="75">
+        <f> 1546936 + 2700897 + 579935</f>
+        <v>4827768</v>
+      </c>
+      <c r="E19" s="75">
+        <f> 2026592 + 852012 + 170320</f>
+        <v>3048924</v>
+      </c>
+      <c r="F19" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G19" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H19" s="76" t="str">
+        <v>7876692</v>
+      </c>
+      <c r="H19" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>206.7427492</v>
       </c>
       <c r="I19" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>42.17552083</v>
       </c>
       <c r="J19" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V19" s="15"/>
       <c r="W19" s="15"/>
@@ -55178,25 +55591,34 @@
       <c r="B20" s="39">
         <v>46095.0</v>
       </c>
-      <c r="C20" s="56"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="56"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="56" t="str">
+      <c r="C20" s="75">
+        <v>38499.0</v>
+      </c>
+      <c r="D20" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="E20" s="75">
+        <f> 1886119 + 475758 + 652933</f>
+        <v>3014810</v>
+      </c>
+      <c r="F20" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G20" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H20" s="76" t="str">
+        <v>3014810</v>
+      </c>
+      <c r="H20" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>78.30878724</v>
       </c>
       <c r="I20" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>15.9749926</v>
       </c>
       <c r="J20" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V20" s="15"/>
       <c r="W20" s="15"/>
@@ -55206,25 +55628,34 @@
       <c r="B21" s="39">
         <v>46096.0</v>
       </c>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56" t="str">
+      <c r="C21" s="75">
+        <v>37900.0</v>
+      </c>
+      <c r="D21" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="E21" s="75">
+        <f> 1975845 + 1035061</f>
+        <v>3010906</v>
+      </c>
+      <c r="F21" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G21" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H21" s="76" t="str">
+        <v>3010906</v>
+      </c>
+      <c r="H21" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>79.44343008</v>
       </c>
       <c r="I21" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>16.20645974</v>
       </c>
       <c r="J21" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V21" s="15"/>
       <c r="W21" s="15"/>
@@ -55234,25 +55665,35 @@
       <c r="B22" s="39">
         <v>46097.0</v>
       </c>
-      <c r="C22" s="56"/>
-      <c r="D22" s="56"/>
-      <c r="E22" s="56"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56" t="str">
+      <c r="C22" s="75">
+        <v>39000.0</v>
+      </c>
+      <c r="D22" s="75">
+        <f> 2486527 + 2303716 + 1849927</f>
+        <v>6640170</v>
+      </c>
+      <c r="E22" s="56">
+        <f> 803013 + 399194 + 447648 + 1509043</f>
+        <v>3158898</v>
+      </c>
+      <c r="F22" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G22" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H22" s="76" t="str">
+        <v>9799068</v>
+      </c>
+      <c r="H22" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>251.2581538</v>
       </c>
       <c r="I22" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>51.25666338</v>
       </c>
       <c r="J22" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V22" s="15"/>
       <c r="W22" s="15"/>
@@ -55262,25 +55703,35 @@
       <c r="B23" s="39">
         <v>46098.0</v>
       </c>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56" t="str">
+      <c r="C23" s="75">
+        <v>38798.0</v>
+      </c>
+      <c r="D23" s="75">
+        <f> 1849473 + 2268903 + 1638113</f>
+        <v>5756489</v>
+      </c>
+      <c r="E23" s="75">
+        <f> 1478170 + 957265 + 365580</f>
+        <v>2801015</v>
+      </c>
+      <c r="F23" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G23" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H23" s="76" t="str">
+        <v>8557504</v>
+      </c>
+      <c r="H23" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>220.5655962</v>
       </c>
       <c r="I23" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>44.99538162</v>
       </c>
       <c r="J23" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V23" s="15"/>
       <c r="W23" s="15"/>
@@ -55290,25 +55741,35 @@
       <c r="B24" s="39">
         <v>46099.0</v>
       </c>
-      <c r="C24" s="56"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="56" t="str">
+      <c r="C24" s="75">
+        <v>38000.0</v>
+      </c>
+      <c r="D24" s="75">
+        <f> 2067247 + 1911185 + 1411664 + 534935</f>
+        <v>5925031</v>
+      </c>
+      <c r="E24" s="75">
+        <f> 1287719</f>
+        <v>1287719</v>
+      </c>
+      <c r="F24" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G24" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H24" s="76" t="str">
+        <v>7212750</v>
+      </c>
+      <c r="H24" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>189.8092105</v>
       </c>
       <c r="I24" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>38.72107895</v>
       </c>
       <c r="J24" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="N24" s="1"/>
       <c r="V24" s="15"/>
@@ -55319,25 +55780,34 @@
       <c r="B25" s="39">
         <v>46100.0</v>
       </c>
-      <c r="C25" s="75"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="75"/>
-      <c r="F25" s="75"/>
-      <c r="G25" s="56" t="str">
+      <c r="C25" s="75">
+        <v>38499.0</v>
+      </c>
+      <c r="D25" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="E25" s="75">
+        <f> 1468000 + 131000 + 1100000</f>
+        <v>2699000</v>
+      </c>
+      <c r="F25" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G25" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H25" s="76" t="str">
+        <v>2699000</v>
+      </c>
+      <c r="H25" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>70.10571703</v>
       </c>
       <c r="I25" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>14.30156627</v>
       </c>
       <c r="J25" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V25" s="15"/>
       <c r="W25" s="15"/>
@@ -55347,25 +55817,35 @@
       <c r="B26" s="39">
         <v>46101.0</v>
       </c>
-      <c r="C26" s="75"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="56"/>
-      <c r="F26" s="75"/>
-      <c r="G26" s="56" t="str">
+      <c r="C26" s="75">
+        <v>38499.0</v>
+      </c>
+      <c r="D26" s="75">
+        <f> 1917325 + 1402623</f>
+        <v>3319948</v>
+      </c>
+      <c r="E26" s="75">
+        <f> 970256 + 675574 + 1114271</f>
+        <v>2760101</v>
+      </c>
+      <c r="F26" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G26" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H26" s="76" t="str">
+        <v>6080049</v>
+      </c>
+      <c r="H26" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>157.9274527</v>
       </c>
       <c r="I26" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>32.21720034</v>
       </c>
       <c r="J26" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V26" s="15"/>
       <c r="W26" s="15"/>
@@ -55375,25 +55855,35 @@
       <c r="B27" s="39">
         <v>46102.0</v>
       </c>
-      <c r="C27" s="75"/>
-      <c r="D27" s="75"/>
-      <c r="E27" s="75"/>
-      <c r="F27" s="75"/>
-      <c r="G27" s="56" t="str">
+      <c r="C27" s="75">
+        <v>39089.0</v>
+      </c>
+      <c r="D27" s="75">
+        <f> 1885805 + 2266267 + 2033456</f>
+        <v>6185528</v>
+      </c>
+      <c r="E27" s="75">
+        <f> 1198329 + 1111696 + 1272996</f>
+        <v>3583021</v>
+      </c>
+      <c r="F27" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G27" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H27" s="76" t="str">
+        <v>9768549</v>
+      </c>
+      <c r="H27" s="76">
         <f t="shared" si="2"/>
-        <v/>
+        <v>249.9053186</v>
       </c>
       <c r="I27" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>50.980685</v>
       </c>
       <c r="J27" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V27" s="15"/>
       <c r="W27" s="15"/>
@@ -55403,25 +55893,35 @@
       <c r="B28" s="39">
         <v>46103.0</v>
       </c>
-      <c r="C28" s="75"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="56"/>
-      <c r="F28" s="75"/>
-      <c r="G28" s="56" t="str">
+      <c r="C28" s="75">
+        <v>37499.0</v>
+      </c>
+      <c r="D28" s="75">
+        <f> 3325939 + 2371038 + 1486317</f>
+        <v>7183294</v>
+      </c>
+      <c r="E28" s="75">
+        <f> 997321 + 589056</f>
+        <v>1586377</v>
+      </c>
+      <c r="F28" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G28" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H28" s="104" t="str">
+        <v>8769671</v>
+      </c>
+      <c r="H28" s="104">
         <f t="shared" si="2"/>
-        <v/>
+        <v>233.8641297</v>
       </c>
       <c r="I28" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>47.70828246</v>
       </c>
       <c r="J28" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="N28" s="1"/>
       <c r="V28" s="15"/>
@@ -55432,25 +55932,35 @@
       <c r="B29" s="39">
         <v>46104.0</v>
       </c>
-      <c r="C29" s="75"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="56"/>
-      <c r="F29" s="75"/>
-      <c r="G29" s="56" t="str">
+      <c r="C29" s="75">
+        <v>38400.0</v>
+      </c>
+      <c r="D29" s="75">
+        <f> 2288248 + 1454530 + 642926 + 1093751</f>
+        <v>5479455</v>
+      </c>
+      <c r="E29" s="75">
+        <f> 650780 + 1125386</f>
+        <v>1776166</v>
+      </c>
+      <c r="F29" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G29" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H29" s="104" t="str">
+        <v>7255621</v>
+      </c>
+      <c r="H29" s="104">
         <f t="shared" si="2"/>
-        <v/>
+        <v>188.9484635</v>
       </c>
       <c r="I29" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>38.54548656</v>
       </c>
       <c r="J29" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V29" s="15"/>
       <c r="W29" s="15"/>
@@ -55460,25 +55970,35 @@
       <c r="B30" s="39">
         <v>46105.0</v>
       </c>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="56" t="str">
+      <c r="C30" s="75">
+        <v>38780.0</v>
+      </c>
+      <c r="D30" s="75">
+        <f> 1779292 + 1620011 + 1536063</f>
+        <v>4935366</v>
+      </c>
+      <c r="E30" s="75">
+        <f> 1176452</f>
+        <v>1176452</v>
+      </c>
+      <c r="F30" s="75">
+        <v>1102015.0</v>
+      </c>
+      <c r="G30" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H30" s="104" t="str">
+        <v>7213833</v>
+      </c>
+      <c r="H30" s="104">
         <f t="shared" si="2"/>
-        <v/>
+        <v>186.0194172</v>
       </c>
       <c r="I30" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>37.94796111</v>
       </c>
       <c r="J30" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V30" s="15"/>
       <c r="W30" s="15"/>
@@ -55488,25 +56008,35 @@
       <c r="B31" s="39">
         <v>46106.0</v>
       </c>
-      <c r="C31" s="56"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="56"/>
-      <c r="F31" s="56"/>
-      <c r="G31" s="56" t="str">
+      <c r="C31" s="75">
+        <v>38389.0</v>
+      </c>
+      <c r="D31" s="75">
+        <f> 1765893 + 1601477 + 1290000 + 2213357</f>
+        <v>6870727</v>
+      </c>
+      <c r="E31" s="75">
+        <f> 1033000</f>
+        <v>1033000</v>
+      </c>
+      <c r="F31" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G31" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H31" s="104" t="str">
+        <v>7903727</v>
+      </c>
+      <c r="H31" s="104">
         <f t="shared" si="2"/>
-        <v/>
+        <v>205.8852015</v>
       </c>
       <c r="I31" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>42.0005811</v>
       </c>
       <c r="J31" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V31" s="15"/>
       <c r="W31" s="15"/>
@@ -55516,25 +56046,35 @@
       <c r="B32" s="39">
         <v>46107.0</v>
       </c>
-      <c r="C32" s="56"/>
-      <c r="D32" s="56"/>
-      <c r="E32" s="56"/>
-      <c r="F32" s="56"/>
-      <c r="G32" s="56" t="str">
+      <c r="C32" s="75">
+        <v>38389.0</v>
+      </c>
+      <c r="D32" s="75">
+        <f> 1432160 + 2032074</f>
+        <v>3464234</v>
+      </c>
+      <c r="E32" s="56">
+        <f> 1930940 + 1073563</f>
+        <v>3004503</v>
+      </c>
+      <c r="F32" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G32" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H32" s="104" t="str">
+        <v>6468737</v>
+      </c>
+      <c r="H32" s="104">
         <f t="shared" si="2"/>
-        <v/>
+        <v>168.5049624</v>
       </c>
       <c r="I32" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>34.37501232</v>
       </c>
       <c r="J32" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V32" s="15"/>
       <c r="W32" s="15"/>
@@ -55544,25 +56084,35 @@
       <c r="B33" s="39">
         <v>46108.0</v>
       </c>
-      <c r="C33" s="56"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="56"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56" t="str">
+      <c r="C33" s="75">
+        <v>39200.0</v>
+      </c>
+      <c r="D33" s="75">
+        <f> 1814408 + 767095 + 2290636</f>
+        <v>4872139</v>
+      </c>
+      <c r="E33" s="75">
+        <f> 1551609 + 762064 + 588747</f>
+        <v>2902420</v>
+      </c>
+      <c r="F33" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G33" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H33" s="104" t="str">
+        <v>7774559</v>
+      </c>
+      <c r="H33" s="104">
         <f t="shared" si="2"/>
-        <v/>
+        <v>198.3305867</v>
       </c>
       <c r="I33" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>40.45943969</v>
       </c>
       <c r="J33" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V33" s="15"/>
       <c r="W33" s="15"/>
@@ -55572,25 +56122,34 @@
       <c r="B34" s="39">
         <v>46109.0</v>
       </c>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56" t="str">
+      <c r="C34" s="75">
+        <v>39188.0</v>
+      </c>
+      <c r="D34" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="E34" s="75">
+        <f> 1285390 + 1597669</f>
+        <v>2883059</v>
+      </c>
+      <c r="F34" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G34" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H34" s="104" t="str">
+        <v>2883059</v>
+      </c>
+      <c r="H34" s="104">
         <f t="shared" si="2"/>
-        <v/>
+        <v>73.56994488</v>
       </c>
       <c r="I34" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>15.00826876</v>
       </c>
       <c r="J34" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V34" s="15"/>
       <c r="W34" s="15"/>
@@ -55599,17 +56158,35 @@
       <c r="B35" s="39">
         <v>46110.0</v>
       </c>
-      <c r="G35" s="56" t="str">
+      <c r="C35" s="75">
+        <v>39164.0</v>
+      </c>
+      <c r="D35" s="75">
+        <f> 428136 + 55482 + 390406</f>
+        <v>874024</v>
+      </c>
+      <c r="E35" s="75">
+        <f> 1711227 + 1110293</f>
+        <v>2821520</v>
+      </c>
+      <c r="F35" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G35" s="56">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3695544</v>
+      </c>
+      <c r="H35" s="104">
+        <f t="shared" si="2"/>
+        <v>94.36073945</v>
       </c>
       <c r="I35" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>19.24959085</v>
       </c>
       <c r="J35" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V35" s="15"/>
       <c r="W35" s="15"/>
@@ -55618,21 +56195,35 @@
       <c r="B36" s="39">
         <v>46111.0</v>
       </c>
-      <c r="G36" s="56" t="str">
+      <c r="C36" s="75">
+        <v>39070.0</v>
+      </c>
+      <c r="D36" s="75">
+        <f> 1583021 + 1959962 + 1932240 + 751731</f>
+        <v>6226954</v>
+      </c>
+      <c r="E36" s="75">
+        <f> 1749014 + 1258488</f>
+        <v>3007502</v>
+      </c>
+      <c r="F36" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G36" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H36" s="104" t="str">
-        <f>IFERROR(G35/C35, )</f>
-        <v/>
+        <v>9234456</v>
+      </c>
+      <c r="H36" s="104">
+        <f t="shared" si="2"/>
+        <v>236.3566931</v>
       </c>
       <c r="I36" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>48.2167654</v>
       </c>
       <c r="J36" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V36" s="15"/>
       <c r="W36" s="15"/>
@@ -55641,21 +56232,35 @@
       <c r="B37" s="39">
         <v>46112.0</v>
       </c>
-      <c r="G37" s="56" t="str">
+      <c r="C37" s="75">
+        <v>38399.0</v>
+      </c>
+      <c r="D37" s="75">
+        <f> 2272686 + 1253537 + 581213 + 508729</f>
+        <v>4616165</v>
+      </c>
+      <c r="E37" s="75">
+        <f> 1643998 + 1393955</f>
+        <v>3037953</v>
+      </c>
+      <c r="F37" s="75">
+        <v>0.0</v>
+      </c>
+      <c r="G37" s="56">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H37" s="104" t="str">
-        <f>IFERROR(G37/C37, )</f>
-        <v/>
+        <v>7654118</v>
+      </c>
+      <c r="H37" s="104">
+        <f t="shared" si="2"/>
+        <v>199.3311805</v>
       </c>
       <c r="I37" s="77">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>40.66356082</v>
       </c>
       <c r="J37" s="41" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Sim</v>
       </c>
       <c r="V37" s="15"/>
       <c r="W37" s="15"/>
@@ -60491,7 +61096,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C34">
+  <conditionalFormatting sqref="C6:C37">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="percent" val="0"/>
@@ -60587,7 +61192,9 @@
       <c r="B3" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="70"/>
+      <c r="C3" s="70">
+        <v>51.0</v>
+      </c>
       <c r="J3" s="15"/>
       <c r="V3" s="15"/>
       <c r="W3" s="15"/>
@@ -60596,7 +61203,9 @@
       <c r="B4" s="69" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="71"/>
+      <c r="C4" s="71">
+        <v>5000.0</v>
+      </c>
       <c r="J4" s="15"/>
       <c r="V4" s="15"/>
       <c r="W4" s="15"/>
@@ -60654,7 +61263,9 @@
       <c r="B7" s="39">
         <v>46113.0</v>
       </c>
-      <c r="C7" s="75"/>
+      <c r="C7" s="75">
+        <v>38396.0</v>
+      </c>
       <c r="D7" s="75"/>
       <c r="E7" s="75"/>
       <c r="F7" s="75"/>
@@ -60662,9 +61273,9 @@
         <f t="shared" ref="G7:G36" si="1">IF(SUM(D7:F7) = 0, , (SUM(D7:F7)))</f>
         <v/>
       </c>
-      <c r="H7" s="76" t="str">
-        <f t="shared" ref="H7:H34" si="2">IFERROR(G7/C7, )</f>
-        <v/>
+      <c r="H7" s="76">
+        <f t="shared" ref="H7:H36" si="2">IFERROR(G7/C7, )</f>
+        <v>0</v>
       </c>
       <c r="I7" s="77">
         <f t="shared" ref="I7:I36" si="3">IFERROR(H7/25 * ($C$3/10), )</f>
@@ -60673,7 +61284,7 @@
       <c r="J7" s="41" t="str">
         <f t="shared" ref="J7:J36" si="4">IF(B7 &gt; TODAY(), "", IF(G7 = "", "Não", "Sim"))
 </f>
-        <v/>
+        <v>Não</v>
       </c>
       <c r="L7" s="78"/>
       <c r="M7" s="79" t="s">
@@ -60724,9 +61335,9 @@
       <c r="L8" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="M8" s="85" t="str">
+      <c r="M8" s="85">
         <f> IFERROR(MEDIAN(C7:C998), )</f>
-        <v/>
+        <v>38396</v>
       </c>
       <c r="N8" s="86"/>
       <c r="O8" s="87"/>
@@ -60777,9 +61388,9 @@
         <f t="shared" ref="M9:N9" si="5"> IFERROR(MEDIAN(G7:G998), )</f>
         <v/>
       </c>
-      <c r="N9" s="56" t="str">
+      <c r="N9" s="56">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O9" s="93">
         <f> IFERROR($N$9 * ($C$3/10)  / 25, )</f>
@@ -60832,9 +61443,9 @@
         <f>IFERROR(SUM(G7:G998), )</f>
         <v>0</v>
       </c>
-      <c r="N10" s="95" t="str">
+      <c r="N10" s="95">
         <f> IFERROR($M$10 / $M$8, )</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O10" s="93">
         <f> IFERROR($N$10 * ($C$3/10)  / 25, )</f>
@@ -60885,22 +61496,22 @@
       </c>
       <c r="M11" s="75">
         <f> IFERROR($N$11 * $M$8, )</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="98" t="str">
+        <v>191980000</v>
+      </c>
+      <c r="N11" s="98">
         <f> IFERROR($C$4, )</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="O11" s="93">
         <f> IFERROR($N$11 * ($C$3/10)  / 25,"")</f>
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="Q11" s="89" t="s">
         <v>62</v>
       </c>
       <c r="R11" s="17">
         <f>COUNTIF($J:$J, "=Não")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11" s="90"/>
       <c r="U11" s="91"/>
@@ -60939,15 +61550,15 @@
       </c>
       <c r="M12" s="56">
         <f> IFERROR($M$11 - $M$10, )</f>
-        <v>0</v>
+        <v>191980000</v>
       </c>
       <c r="N12" s="56">
         <f>N11 - N10</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="O12" s="93">
         <f> IFERROR($N$12 * ($C$3/10)  / 25, )</f>
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="Q12" s="89" t="s">
         <v>64</v>
@@ -60997,7 +61608,7 @@
       </c>
       <c r="R13" s="23" t="str">
         <f>IF(M10 &gt;= M11, "🔵 Concluído", IF((R8-R9)-R10-R11&gt;=2, "🟢 Seguro", IF((R8-R9)-R10-R11&gt;=0, "🟡 Atenção", "🔴 Risco")))</f>
-        <v>🔵 Concluído</v>
+        <v>🟢 Seguro</v>
       </c>
       <c r="T13" s="90"/>
       <c r="U13" s="91"/>
@@ -61613,6 +62224,10 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
+      <c r="H35" s="104" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
       <c r="I35" s="77">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -61633,7 +62248,7 @@
         <v/>
       </c>
       <c r="H36" s="104" t="str">
-        <f>IFERROR(G35/C35, )</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="I36" s="77">

</xml_diff>